<commit_message>
modification majeur de ma fonction generate_export
</commit_message>
<xml_diff>
--- a/data/rapport_velib.xlsx
+++ b/data/rapport_velib.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,10 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000000FF"/>
     </font>
     <font>
       <b val="1"/>
@@ -57,12 +61,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -283,6 +288,7 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -293,7 +299,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Top 5 des communes (Moyenne vélos disponibles)</a:t>
+              <a:t>Nombre de vélo par occupation dans chaque commune du top</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -301,7 +307,7 @@
     </title>
     <plotArea>
       <barChart>
-        <barDir val="bar"/>
+        <barDir val="col"/>
         <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
@@ -326,6 +332,33 @@
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Indicateurs'!$C$18:$C$22</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -341,7 +374,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Moyenne</a:t>
+                  <a:t>Communes</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -359,9 +392,51 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Nombre moyen de vélos</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Taux d'occupation en (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -396,12 +471,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>13</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="5400000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -420,10 +495,10 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="5400000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -96019,18 +96094,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B22"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Choisir une commune :</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>TABLEAU DE BORD DU RÉSEAU VÉLIB</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Indicateurs Réseau</t>
         </is>
@@ -96043,7 +96130,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>SUM(DATA!D2:D1512)</f>
+        <f>SUMIF(DATA!M2:M1512, B1, DATA!D2:D1512)</f>
         <v/>
       </c>
     </row>
@@ -96054,7 +96141,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>SUM(DATA!E2:E1512)</f>
+        <f>SUMIF(DATA!M2:M1512, B1, DATA!E2:E1512)</f>
         <v/>
       </c>
     </row>
@@ -96065,7 +96152,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>SUM(DATA!F2:F1512)</f>
+        <f>SUMIF(DATA!M2:M1512, B1, DATA!F2:F1512)</f>
         <v/>
       </c>
     </row>
@@ -96075,13 +96162,13 @@
           <t>Taux d'occupation global</t>
         </is>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="6">
         <f>B7/B5</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Répartition par type de vélo</t>
         </is>
@@ -96094,7 +96181,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>SUM(DATA!G2:G1512)</f>
+        <f>SUMIF(DATA!M2:M1512, B1, DATA!G2:G1512)</f>
         <v/>
       </c>
     </row>
@@ -96105,7 +96192,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>SUM(DATA!H2:H1512)</f>
+        <f>SUMIF(DATA!M2:M1512, B1, DATA!H2:H1512)</f>
         <v/>
       </c>
     </row>
@@ -96121,7 +96208,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Top 5 des communes les plus desservies en vélo</t>
         </is>
@@ -96136,6 +96223,9 @@
       <c r="B18" t="n">
         <v>25.8</v>
       </c>
+      <c r="C18" t="n">
+        <v>6358</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -96146,6 +96236,9 @@
       <c r="B19" t="n">
         <v>24.7</v>
       </c>
+      <c r="C19" t="n">
+        <v>7549.7</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -96156,6 +96249,9 @@
       <c r="B20" t="n">
         <v>22</v>
       </c>
+      <c r="C20" t="n">
+        <v>5500</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -96166,6 +96262,9 @@
       <c r="B21" t="n">
         <v>21</v>
       </c>
+      <c r="C21" t="n">
+        <v>6855.2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -96176,8 +96275,16 @@
       <c r="B22" t="n">
         <v>20.4</v>
       </c>
+      <c r="C22" t="n">
+        <v>5640.5</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Saisie invalide" error="Votre commune n'est pas dans la liste" promptTitle="Liste des communes" prompt="SVP choisissez une commune dans la liste" type="list">
+      <formula1>"Alfortville,Arcueil,Argenteuil,Asnières-sur-Seine,Aubervilliers,Bagneux,Bagnolet,Bobigny,Bois-Colombes,Boulogne-Billancourt,Bourg-la-Reine,Cachan,Champigny-sur-Marne,Charenton-le-Pont,Chaville,Chevilly-Larue,Choisy-le-Roi,Châtillon,Clamart,Clichy,Colombes,Courbevoie,Créteil,Fontenay-aux-Roses,Fontenay-sous-Bois,Garches,Gennevilliers,Gentilly,Issy-les-Moulineaux,Ivry-sur-Seine,Joinville-le-Pont,L'Île-Saint-Denis,La Courneuve,La Garenne-Colombes,Le Kremlin-Bicêtre,Le Pré-Saint-Gervais,Les Lilas,Levallois-Perret,Maisons-Alfort,Malakoff,Meudon,Montreuil,Montrouge,Nanterre,Neuilly-sur-Seine,Nogent-sur-Marne,Noisy-le-Sec,Orly,Pantin,Paris,Puteaux,Romainville,Rosny-sous-Bois,Rueil-Malmaison,Saint-Cloud,Saint-Denis,Saint-Mandé,Saint-Maurice,Saint-Ouen-sur-Seine,Sceaux,Suresnes,Sèvres,Thiais,Vanves,Ville-d'Avray,Villejuif,Villeneuve-la-Garenne,Vincennes,Vitry-sur-Seine"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
mon filtre ne fonctionne pas à revoir
</commit_message>
<xml_diff>
--- a/data/rapport_velib.xlsx
+++ b/data/rapport_velib.xlsx
@@ -288,6 +288,95 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Top 5 des communes (Moyenne vélos disponibles)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Indicateurs'!$A$18:$A$22</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Indicateurs'!$B$18:$B$22</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Moyenne</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
@@ -495,7 +584,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="4320000"/>
@@ -508,6 +597,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -96094,7 +96205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -96108,6 +96219,16 @@
           <t>Paris</t>
         </is>
       </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Choisir une station :</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Abbeville - Faubourg Poissonnière</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -96280,9 +96401,12 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Saisie invalide" error="Votre commune n'est pas dans la liste" promptTitle="Liste des communes" prompt="SVP choisissez une commune dans la liste" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="B1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alfortville,Arcueil,Argenteuil,Asnières-sur-Seine,Aubervilliers,Bagneux,Bagnolet,Bobigny,Bois-Colombes,Boulogne-Billancourt,Bourg-la-Reine,Cachan,Champigny-sur-Marne,Charenton-le-Pont,Chaville,Chevilly-Larue,Choisy-le-Roi,Châtillon,Clamart,Clichy,Colombes,Courbevoie,Créteil,Fontenay-aux-Roses,Fontenay-sous-Bois,Garches,Gennevilliers,Gentilly,Issy-les-Moulineaux,Ivry-sur-Seine,Joinville-le-Pont,L'Île-Saint-Denis,La Courneuve,La Garenne-Colombes,Le Kremlin-Bicêtre,Le Pré-Saint-Gervais,Les Lilas,Levallois-Perret,Maisons-Alfort,Malakoff,Meudon,Montreuil,Montrouge,Nanterre,Neuilly-sur-Seine,Nogent-sur-Marne,Noisy-le-Sec,Orly,Pantin,Paris,Puteaux,Romainville,Rosny-sous-Bois,Rueil-Malmaison,Saint-Cloud,Saint-Denis,Saint-Mandé,Saint-Maurice,Saint-Ouen-sur-Seine,Sceaux,Suresnes,Sèvres,Thiais,Vanves,Ville-d'Avray,Villejuif,Villeneuve-la-Garenne,Vincennes,Vitry-sur-Seine"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DATA!$B$2:$B$1512</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
insert° de la carte dans le rapport
</commit_message>
<xml_diff>
--- a/data/rapport_velib.xlsx
+++ b/data/rapport_velib.xlsx
@@ -30,7 +30,8 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="14"/>
+      <color rgb="001F497D"/>
+      <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
@@ -288,95 +289,6 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Top 5 des communes (Moyenne vélos disponibles)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Indicateurs'!$A$18:$A$22</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Indicateurs'!$B$18:$B$22</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Moyenne</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
@@ -584,7 +496,7 @@
     <from>
       <col>4</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="4320000"/>
@@ -604,24 +516,27 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>13</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="4320000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="4" name="Chart 4"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="5238750" cy="3810000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>
@@ -96205,7 +96120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -96219,19 +96134,9 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Choisir une station :</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Abbeville - Faubourg Poissonnière</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>TABLEAU DE BORD DU RÉSEAU VÉLIB</t>
         </is>
@@ -96401,12 +96306,9 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation sqref="B1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alfortville,Arcueil,Argenteuil,Asnières-sur-Seine,Aubervilliers,Bagneux,Bagnolet,Bobigny,Bois-Colombes,Boulogne-Billancourt,Bourg-la-Reine,Cachan,Champigny-sur-Marne,Charenton-le-Pont,Chaville,Chevilly-Larue,Choisy-le-Roi,Châtillon,Clamart,Clichy,Colombes,Courbevoie,Créteil,Fontenay-aux-Roses,Fontenay-sous-Bois,Garches,Gennevilliers,Gentilly,Issy-les-Moulineaux,Ivry-sur-Seine,Joinville-le-Pont,L'Île-Saint-Denis,La Courneuve,La Garenne-Colombes,Le Kremlin-Bicêtre,Le Pré-Saint-Gervais,Les Lilas,Levallois-Perret,Maisons-Alfort,Malakoff,Meudon,Montreuil,Montrouge,Nanterre,Neuilly-sur-Seine,Nogent-sur-Marne,Noisy-le-Sec,Orly,Pantin,Paris,Puteaux,Romainville,Rosny-sous-Bois,Rueil-Malmaison,Saint-Cloud,Saint-Denis,Saint-Mandé,Saint-Maurice,Saint-Ouen-sur-Seine,Sceaux,Suresnes,Sèvres,Thiais,Vanves,Ville-d'Avray,Villejuif,Villeneuve-la-Garenne,Vincennes,Vitry-sur-Seine"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F1" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>DATA!$B$2:$B$1512</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>